<commit_message>
Bake cached values into consistency-check xlsx (formulas + values)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ye6aaquAcEaEzL9cvV7wY
</commit_message>
<xml_diff>
--- a/数据一致性核对_2026-07.xlsx
+++ b/数据一致性核对_2026-07.xlsx
@@ -630,9 +630,10 @@
           <t>① MTD Cost</t>
         </is>
       </c>
-      <c r="B4" s="4">
-        <f> Action Earnings + AF Cost   ⟹   Action Earnings = MTD Cost − AF Cost</f>
-        <v/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>MTD Cost = Action Earnings + AF Cost　（⟹ Action Earnings = MTD Cost − AF Cost）</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -641,9 +642,10 @@
           <t>② 核减金额</t>
         </is>
       </c>
-      <c r="B5" s="4">
-        <f> AF Cost − (AF Cost + Action Earnings) × 优化目标%  = AF Cost − MTD Cost × 优化目标%</f>
-        <v/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>核减金额 = AF Cost − (AF Cost + Action Earnings) × 优化目标%　= AF Cost − MTD Cost × 优化目标%</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -652,9 +654,10 @@
           <t>③ AF Cost%</t>
         </is>
       </c>
-      <c r="B6" s="4">
-        <f> AF Cost / MTD Cost</f>
-        <v/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>AF Cost% = AF Cost / MTD Cost</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -937,15 +940,15 @@
       </c>
       <c r="H3" s="14">
         <f>G3-F3</f>
-        <v/>
+        <v>8379</v>
       </c>
       <c r="I3" s="15">
         <f>IF(G3=0,0,F3/G3)</f>
-        <v/>
+        <v>0.1127700127</v>
       </c>
       <c r="J3" s="14">
         <f>F3-G3*E3</f>
-        <v/>
+        <v>120.6</v>
       </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
@@ -985,15 +988,15 @@
       </c>
       <c r="H4" s="14">
         <f>G4-F4</f>
-        <v/>
+        <v>4447</v>
       </c>
       <c r="I4" s="15">
         <f>IF(G4=0,0,F4/G4)</f>
-        <v/>
+        <v>0.2101243339</v>
       </c>
       <c r="J4" s="14">
         <f>F4-G4*E4</f>
-        <v/>
+        <v>620</v>
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
@@ -1013,23 +1016,23 @@
       <c r="E5" s="17" t="n"/>
       <c r="F5" s="18">
         <f>SUM(F3:F4)</f>
-        <v/>
+        <v>2248</v>
       </c>
       <c r="G5" s="18">
         <f>SUM(G3:G4)</f>
-        <v/>
+        <v>15074</v>
       </c>
       <c r="H5" s="18">
         <f>SUM(H3:H4)</f>
-        <v/>
+        <v>12826</v>
       </c>
       <c r="I5" s="19">
         <f>IF(G5=0,0,F5/G5)</f>
-        <v/>
+        <v>0.149130954</v>
       </c>
       <c r="J5" s="18">
         <f>SUM(J3:J4)</f>
-        <v/>
+        <v>740.6</v>
       </c>
       <c r="K5" s="17" t="n"/>
     </row>
@@ -1173,15 +1176,15 @@
       </c>
       <c r="H3" s="14">
         <f>G3-F3</f>
-        <v/>
+        <v>32365</v>
       </c>
       <c r="I3" s="15">
         <f>IF(G3=0,0,F3/G3)</f>
-        <v/>
+        <v>0.1081565169</v>
       </c>
       <c r="J3" s="14">
         <f>F3-G3*E3</f>
-        <v/>
+        <v>-1518.5</v>
       </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
@@ -1221,15 +1224,15 @@
       </c>
       <c r="H4" s="14">
         <f>G4-F4</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I4" s="15">
         <f>IF(G4=0,0,F4/G4)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J4" s="14">
         <f>F4-G4*E4</f>
-        <v/>
+        <v>10.2</v>
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
@@ -1269,15 +1272,15 @@
       </c>
       <c r="H5" s="14">
         <f>G5-F5</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I5" s="15">
         <f>IF(G5=0,0,F5/G5)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J5" s="14">
         <f>F5-G5*E5</f>
-        <v/>
+        <v>5.1</v>
       </c>
       <c r="K5" s="9" t="inlineStr">
         <is>
@@ -1317,15 +1320,15 @@
       </c>
       <c r="H6" s="14">
         <f>G6-F6</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I6" s="15">
         <f>IF(G6=0,0,F6/G6)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J6" s="14">
         <f>F6-G6*E6</f>
-        <v/>
+        <v>3.4</v>
       </c>
       <c r="K6" s="9" t="inlineStr">
         <is>
@@ -1345,23 +1348,23 @@
       <c r="E7" s="17" t="n"/>
       <c r="F7" s="18">
         <f>SUM(F3:F6)</f>
-        <v/>
+        <v>3947</v>
       </c>
       <c r="G7" s="18">
         <f>SUM(G3:G6)</f>
-        <v/>
+        <v>36312</v>
       </c>
       <c r="H7" s="18">
         <f>SUM(H3:H6)</f>
-        <v/>
+        <v>32365</v>
       </c>
       <c r="I7" s="19">
         <f>IF(G7=0,0,F7/G7)</f>
-        <v/>
+        <v>0.1086968495</v>
       </c>
       <c r="J7" s="18">
         <f>SUM(J3:J6)</f>
-        <v/>
+        <v>-1499.8</v>
       </c>
       <c r="K7" s="17" t="n"/>
     </row>
@@ -1391,7 +1394,7 @@
       </c>
       <c r="H11" s="23">
         <f>H7</f>
-        <v/>
+        <v>32365</v>
       </c>
     </row>
     <row r="12">
@@ -1402,11 +1405,11 @@
       </c>
       <c r="H12" s="24">
         <f>H11-H10</f>
-        <v/>
-      </c>
-      <c r="I12" s="3">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3" t="str">
         <f>IF(ABS(H12)&lt;0.5,"✅ 一致","⚠️ 不一致")</f>
-        <v/>
+        <v>✅ 一致</v>
       </c>
     </row>
   </sheetData>
@@ -1698,19 +1701,19 @@
       <c r="B12" s="17" t="n"/>
       <c r="C12" s="28">
         <f>SUM(C3:C11)</f>
-        <v/>
+        <v>1351448</v>
       </c>
       <c r="D12" s="28">
         <f>SUM(D3:D11)</f>
-        <v/>
+        <v>326133</v>
       </c>
       <c r="E12" s="29">
         <f>SUM(E3:E11)</f>
-        <v/>
+        <v>1320783.82</v>
       </c>
       <c r="F12" s="29">
         <f>SUM(F3:F11)</f>
-        <v/>
+        <v>12947.18</v>
       </c>
     </row>
     <row r="14">
@@ -1735,7 +1738,7 @@
       </c>
       <c r="F16" s="31">
         <f>SUMIF($B$3:$B$11,"TH",$F$3:$F$11)</f>
-        <v/>
+        <v>8518.64</v>
       </c>
     </row>
     <row r="17">
@@ -1746,7 +1749,7 @@
       </c>
       <c r="F17" s="31">
         <f>SUMIF($B$3:$B$11,"PH",$F$3:$F$11)</f>
-        <v/>
+        <v>4428.54</v>
       </c>
     </row>
     <row r="18">
@@ -1757,7 +1760,7 @@
       </c>
       <c r="F18" s="32">
         <f>SUM(F16:F17)</f>
-        <v/>
+        <v>12947.18</v>
       </c>
     </row>
   </sheetData>
@@ -1813,7 +1816,7 @@
       </c>
       <c r="C4" s="35">
         <f>'4046-CPA核算'!H7</f>
-        <v/>
+        <v>32365</v>
       </c>
     </row>
     <row r="5">
@@ -1834,11 +1837,11 @@
       </c>
       <c r="C6" s="37">
         <f>C4-C5</f>
-        <v/>
-      </c>
-      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="str">
         <f>IF(ABS(C6)&lt;0.5,"✅ 完全一致","⚠️ 不一致")</f>
-        <v/>
+        <v>✅ 完全一致</v>
       </c>
     </row>
     <row r="8">
@@ -1860,7 +1863,7 @@
       </c>
       <c r="C9" s="38">
         <f>'SubId2明细-4696'!F12</f>
-        <v/>
+        <v>12947.18</v>
       </c>
     </row>
     <row r="10">
@@ -1871,7 +1874,7 @@
       </c>
       <c r="C10" s="38">
         <f>'4696-CPS核算'!H5</f>
-        <v/>
+        <v>12826</v>
       </c>
     </row>
     <row r="11">
@@ -1882,7 +1885,7 @@
       </c>
       <c r="C11" s="31">
         <f>C9-C10</f>
-        <v/>
+        <v>121.18</v>
       </c>
       <c r="D11" s="30" t="inlineStr">
         <is>
@@ -1951,31 +1954,31 @@
       </c>
       <c r="B15" s="40">
         <f>'4696-CPS核算'!H3</f>
-        <v/>
+        <v>8379</v>
       </c>
       <c r="C15" s="40">
         <f>'SubId2明细-4696'!F16</f>
-        <v/>
+        <v>8518.64</v>
       </c>
       <c r="D15" s="41">
         <f>B15-C15</f>
-        <v/>
+        <v>-139.64</v>
       </c>
       <c r="E15" s="42">
         <f>C15+'4696-CPS核算'!F3</f>
-        <v/>
+        <v>9583.64</v>
       </c>
       <c r="F15" s="42">
         <f>'4696-CPS核算'!F3-E15*'4696-CPS核算'!E3</f>
-        <v/>
+        <v>106.636</v>
       </c>
       <c r="G15" s="40">
         <f>'4696-CPS核算'!J3</f>
-        <v/>
+        <v>120.6</v>
       </c>
       <c r="H15" s="41">
         <f>G15-F15</f>
-        <v/>
+        <v>13.964</v>
       </c>
     </row>
     <row r="16">
@@ -1986,31 +1989,31 @@
       </c>
       <c r="B16" s="40">
         <f>'4696-CPS核算'!H4</f>
-        <v/>
+        <v>4447</v>
       </c>
       <c r="C16" s="40">
         <f>'SubId2明细-4696'!F17</f>
-        <v/>
+        <v>4428.54</v>
       </c>
       <c r="D16" s="41">
         <f>B16-C16</f>
-        <v/>
+        <v>18.46</v>
       </c>
       <c r="E16" s="42">
         <f>C16+'4696-CPS核算'!F4</f>
-        <v/>
+        <v>5611.54</v>
       </c>
       <c r="F16" s="42">
         <f>'4696-CPS核算'!F4-E16*'4696-CPS核算'!E4</f>
-        <v/>
+        <v>621.846</v>
       </c>
       <c r="G16" s="40">
         <f>'4696-CPS核算'!J4</f>
-        <v/>
+        <v>620</v>
       </c>
       <c r="H16" s="41">
         <f>G16-F16</f>
-        <v/>
+        <v>-1.846</v>
       </c>
     </row>
     <row r="17">
@@ -2021,28 +2024,28 @@
       </c>
       <c r="B17" s="29">
         <f>SUM(B15:B16)</f>
-        <v/>
+        <v>12826</v>
       </c>
       <c r="C17" s="29">
         <f>SUM(C15:C16)</f>
-        <v/>
+        <v>12947.18</v>
       </c>
       <c r="D17" s="29">
         <f>SUM(D15:D16)</f>
-        <v/>
+        <v>-121.18</v>
       </c>
       <c r="E17" s="17" t="n"/>
       <c r="F17" s="29">
         <f>SUM(F15:F16)</f>
-        <v/>
+        <v>728.482</v>
       </c>
       <c r="G17" s="29">
         <f>SUM(G15:G16)</f>
-        <v/>
+        <v>740.6</v>
       </c>
       <c r="H17" s="29">
         <f>SUM(H15:H16)</f>
-        <v/>
+        <v>12.118</v>
       </c>
     </row>
     <row r="19">

</xml_diff>